<commit_message>
wrote a seperate _create_chart method
</commit_message>
<xml_diff>
--- a/100040000/output.xlsx
+++ b/100040000/output.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carla\clariant\mini_project\100040000\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84070CBA-3B0E-47AC-AE6D-E318CEC15C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F02C0C0D-2FF9-4932-A041-89FB8E8D76E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="23985" windowHeight="13650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="200122941" sheetId="1" r:id="rId1"/>
@@ -65,12 +65,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="13">
   <si>
-    <t>Particle</t>
+    <t>Particle (N)</t>
   </si>
   <si>
-    <t>Diameter (nm)</t>
+    <t>Particle Size (nm)</t>
   </si>
   <si>
     <t>min</t>
@@ -104,9 +104,6 @@
   </si>
   <si>
     <t>data_for_mid_calc</t>
-  </si>
-  <si>
-    <t>length</t>
   </si>
 </sst>
 </file>
@@ -346,7 +343,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2767-40DA-AC4C-08CB294076F9}"/>
+              <c16:uniqueId val="{00000000-55F2-4417-BED0-5DEC22F04B37}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -495,7 +492,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-2767-40DA-AC4C-08CB294076F9}"/>
+              <c16:uniqueId val="{00000001-55F2-4417-BED0-5DEC22F04B37}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -784,7 +781,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E494-45F9-ABA6-322657490EE5}"/>
+              <c16:uniqueId val="{00000000-B843-4813-A27F-917E720B351A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -963,7 +960,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-E494-45F9-ABA6-322657490EE5}"/>
+              <c16:uniqueId val="{00000001-B843-4813-A27F-917E720B351A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1258,7 +1255,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8947-4787-97FF-513343D0F8AE}"/>
+              <c16:uniqueId val="{00000000-5AC7-42E9-B465-F57434AC6520}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1443,7 +1440,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-8947-4787-97FF-513343D0F8AE}"/>
+              <c16:uniqueId val="{00000001-5AC7-42E9-B465-F57434AC6520}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1548,15 +1545,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>314325</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>85725</xdr:rowOff>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1588,15 +1585,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1629,16 +1626,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>219075</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>523875</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1953,13 +1950,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R201"/>
+  <dimension ref="A1:Q201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1999,11 +1997,8 @@
       <c r="Q1" t="s">
         <v>12</v>
       </c>
-      <c r="R1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2049,12 +2044,8 @@
         <f t="array" ref="Q2:Q17">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,O2+J2,J2)</f>
         <v>2</v>
       </c>
-      <c r="R2" cm="1">
-        <f t="array" ref="R2">ROWS(_xlfn.ANCHORARRAY(K2))</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2074,7 +2065,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2094,7 +2085,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2114,7 +2105,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2134,7 +2125,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2154,7 +2145,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2174,7 +2165,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2194,7 +2185,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2214,7 +2205,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2234,7 +2225,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2254,7 +2245,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2274,7 +2265,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2294,7 +2285,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2314,7 +2305,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3834,10 +3825,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R201"/>
+  <dimension ref="A1:Q201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3877,11 +3872,8 @@
       <c r="Q1" t="s">
         <v>12</v>
       </c>
-      <c r="R1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3927,12 +3919,8 @@
         <f t="array" ref="Q2:Q22">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,O2+J2,J2)</f>
         <v>5</v>
       </c>
-      <c r="R2" cm="1">
-        <f t="array" ref="R2">ROWS(_xlfn.ANCHORARRAY(K2))</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3952,7 +3940,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3972,7 +3960,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3992,7 +3980,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -4012,7 +4000,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -4032,7 +4020,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -4052,7 +4040,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -4072,7 +4060,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -4092,7 +4080,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -4112,7 +4100,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -4132,7 +4120,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -4152,7 +4140,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -4172,7 +4160,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -4192,7 +4180,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -5772,10 +5760,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:R201"/>
+  <dimension ref="A1:Q201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5815,11 +5808,8 @@
       <c r="Q1" t="s">
         <v>12</v>
       </c>
-      <c r="R1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5865,12 +5855,8 @@
         <f t="array" ref="Q2:Q23">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,O2+J2,J2)</f>
         <v>3</v>
       </c>
-      <c r="R2" cm="1">
-        <f t="array" ref="R2">ROWS(_xlfn.ANCHORARRAY(K2))</f>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -5890,7 +5876,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -5910,7 +5896,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -5930,7 +5916,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -5950,7 +5936,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -5970,7 +5956,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -5990,7 +5976,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -6010,7 +5996,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -6030,7 +6016,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -6050,7 +6036,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -6070,7 +6056,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -6090,7 +6076,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -6110,7 +6096,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -6130,7 +6116,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
saving this instance, might need a macro version
</commit_message>
<xml_diff>
--- a/100040000/output.xlsx
+++ b/100040000/output.xlsx
@@ -18,6 +18,12 @@
     <definedName name="frequencies_200122941">200122941!$M$2:INDEX(200122941!$M:$M,2+COUNT(_xlfn.ANCHORARRAY(200122941!$M$2))-1)</definedName>
     <definedName name="frequencies_200122942">200122942!$M$2:INDEX(200122942!$M:$M,2+COUNT(_xlfn.ANCHORARRAY(200122942!$M$2))-1)</definedName>
     <definedName name="frequencies_200122943">200122943!$M$2:INDEX(200122943!$M:$M,2+COUNT(_xlfn.ANCHORARRAY(200122943!$M$2))-1)</definedName>
+    <definedName name="mid_200122941">200122941!$L$2:INDEX(200122941!$L:$L,2+COUNT(_xlfn.ANCHORARRAY(200122941!$L$2))-1)</definedName>
+    <definedName name="mid_200122942">200122942!$L$2:INDEX(200122942!$L:$L,2+COUNT(_xlfn.ANCHORARRAY(200122942!$L$2))-1)</definedName>
+    <definedName name="mid_200122943">200122943!$L$2:INDEX(200122943!$L:$L,2+COUNT(_xlfn.ANCHORARRAY(200122943!$L$2))-1)</definedName>
+    <definedName name="zeros_200122941">200122941!$R$2:INDEX(200122941!$R:$R,2+COUNT(_xlfn.ANCHORARRAY(200122941!$R$2))-1)</definedName>
+    <definedName name="zeros_200122942">200122942!$R$2:INDEX(200122942!$R:$R,2+COUNT(_xlfn.ANCHORARRAY(200122942!$R$2))-1)</definedName>
+    <definedName name="zeros_200122943">200122943!$R$2:INDEX(200122943!$R:$R,2+COUNT(_xlfn.ANCHORARRAY(200122943!$R$2))-1)</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="14">
   <si>
     <t>Particle (N)</t>
   </si>
@@ -86,6 +92,9 @@
   <si>
     <t>data_for_mid_calc</t>
   </si>
+  <si>
+    <t>zeros</t>
+  </si>
 </sst>
 </file>
 
@@ -109,7 +118,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -155,7 +164,7 @@
   <dxfs count="1">
     <dxf>
       <font>
-        <color rgb="FFFFFFFF"/>
+        <color rgb="FF000000"/>
       </font>
     </dxf>
   </dxfs>
@@ -187,15 +196,39 @@
     </c:title>
     <c:plotArea>
       <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:cat>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:errBars>
+            <c:errDir val="y"/>
+            <c:errBarType val="minus"/>
+            <c:errValType val="percentage"/>
+            <c:noEndCap val="1"/>
+            <c:val val="100"/>
+            <c:spPr>
+              <a:ln w="127000">
+                <a:solidFill>
+                  <a:srgbClr val="ED7D31"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:errBars>
+          <c:xVal>
             <c:strRef>
-              <c:f>200122941!bin_200122941</c:f>
+              <c:f>200122941!mid_200122941</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -203,8 +236,8 @@
                 </c:pt>
               </c:strCache>
             </c:strRef>
-          </c:cat>
-          <c:val>
+          </c:xVal>
+          <c:yVal>
             <c:numRef>
               <c:f>200122941!frequencies_200122941</c:f>
               <c:numCache>
@@ -215,60 +248,18 @@
                 </c:pt>
               </c:numCache>
             </c:numRef>
-          </c:val>
+          </c:yVal>
+          <c:smooth val="1"/>
         </c:ser>
-        <c:gapWidth val="0"/>
         <c:axId val="50010001"/>
         <c:axId val="50010002"/>
-      </c:barChart>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>200122941!bin_200122941</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Particle (N)</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>200122941!frequencies_200122941</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="1"/>
-        </c:ser>
-        <c:marker val="1"/>
-        <c:axId val="50010001"/>
-        <c:axId val="50010002"/>
-      </c:lineChart>
-      <c:catAx>
+      </c:scatterChart>
+      <c:valAx>
         <c:axId val="50010001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="18"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:title>
@@ -289,14 +280,14 @@
           </c:tx>
           <c:layout/>
         </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50010002"/>
         <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-      </c:catAx>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="2"/>
+      </c:valAx>
       <c:valAx>
         <c:axId val="50010002"/>
         <c:scaling>
@@ -307,7 +298,7 @@
         <c:title>
           <c:tx>
             <c:rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="-5400000" vert="horz"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -327,7 +318,7 @@
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50010001"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -364,15 +355,39 @@
     </c:title>
     <c:plotArea>
       <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:cat>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:errBars>
+            <c:errDir val="y"/>
+            <c:errBarType val="minus"/>
+            <c:errValType val="percentage"/>
+            <c:noEndCap val="1"/>
+            <c:val val="100"/>
+            <c:spPr>
+              <a:ln w="152400">
+                <a:solidFill>
+                  <a:srgbClr val="ED7D31"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:errBars>
+          <c:xVal>
             <c:strRef>
-              <c:f>200122942!bin_200122942</c:f>
+              <c:f>200122942!mid_200122942</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -380,8 +395,8 @@
                 </c:pt>
               </c:strCache>
             </c:strRef>
-          </c:cat>
-          <c:val>
+          </c:xVal>
+          <c:yVal>
             <c:numRef>
               <c:f>200122942!frequencies_200122942</c:f>
               <c:numCache>
@@ -392,60 +407,18 @@
                 </c:pt>
               </c:numCache>
             </c:numRef>
-          </c:val>
+          </c:yVal>
+          <c:smooth val="1"/>
         </c:ser>
-        <c:gapWidth val="0"/>
         <c:axId val="50020001"/>
         <c:axId val="50020002"/>
-      </c:barChart>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>200122942!bin_200122942</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Particle (N)</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>200122942!frequencies_200122942</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="1"/>
-        </c:ser>
-        <c:marker val="1"/>
-        <c:axId val="50020001"/>
-        <c:axId val="50020002"/>
-      </c:lineChart>
-      <c:catAx>
+      </c:scatterChart>
+      <c:valAx>
         <c:axId val="50020001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="26"/>
+          <c:min val="4"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:title>
@@ -466,14 +439,14 @@
           </c:tx>
           <c:layout/>
         </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50020002"/>
         <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-      </c:catAx>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="2"/>
+      </c:valAx>
       <c:valAx>
         <c:axId val="50020002"/>
         <c:scaling>
@@ -484,7 +457,7 @@
         <c:title>
           <c:tx>
             <c:rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="-5400000" vert="horz"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -504,7 +477,7 @@
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50020001"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -541,15 +514,39 @@
     </c:title>
     <c:plotArea>
       <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:cat>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:errBars>
+            <c:errDir val="y"/>
+            <c:errBarType val="minus"/>
+            <c:errValType val="percentage"/>
+            <c:noEndCap val="1"/>
+            <c:val val="100"/>
+            <c:spPr>
+              <a:ln w="165100">
+                <a:solidFill>
+                  <a:srgbClr val="ED7D31"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:errBars>
+          <c:xVal>
             <c:strRef>
-              <c:f>200122943!bin_200122943</c:f>
+              <c:f>200122943!mid_200122943</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -557,8 +554,8 @@
                 </c:pt>
               </c:strCache>
             </c:strRef>
-          </c:cat>
-          <c:val>
+          </c:xVal>
+          <c:yVal>
             <c:numRef>
               <c:f>200122943!frequencies_200122943</c:f>
               <c:numCache>
@@ -569,60 +566,18 @@
                 </c:pt>
               </c:numCache>
             </c:numRef>
-          </c:val>
+          </c:yVal>
+          <c:smooth val="1"/>
         </c:ser>
-        <c:gapWidth val="0"/>
         <c:axId val="50030001"/>
         <c:axId val="50030002"/>
-      </c:barChart>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>200122943!bin_200122943</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Particle (N)</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>200122943!frequencies_200122943</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="1"/>
-        </c:ser>
-        <c:marker val="1"/>
-        <c:axId val="50030001"/>
-        <c:axId val="50030002"/>
-      </c:lineChart>
-      <c:catAx>
+      </c:scatterChart>
+      <c:valAx>
         <c:axId val="50030001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="26"/>
+          <c:min val="2"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:title>
@@ -643,14 +598,14 @@
           </c:tx>
           <c:layout/>
         </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50030002"/>
         <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-      </c:catAx>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="2"/>
+      </c:valAx>
       <c:valAx>
         <c:axId val="50030002"/>
         <c:scaling>
@@ -661,7 +616,7 @@
         <c:title>
           <c:tx>
             <c:rich>
-              <a:bodyPr/>
+              <a:bodyPr rot="-5400000" vert="horz"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -681,7 +636,7 @@
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50030001"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -1084,14 +1039,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q201"/>
+  <dimension ref="A1:R201"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1131,8 +1086,11 @@
       <c r="Q1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:17">
+      <c r="R1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1178,8 +1136,12 @@
         <f t="array" ref="Q2">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,O2+J2,J2)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:17">
+      <c r="R2" cm="1">
+        <f t="array" ref="R2">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,0,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1187,7 +1149,7 @@
         <v>4.536</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:18">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1195,7 +1157,7 @@
         <v>9.909000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:18">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1203,7 +1165,7 @@
         <v>6.235</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:18">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1211,7 +1173,7 @@
         <v>9.564</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:18">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1219,7 +1181,7 @@
         <v>9.977</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:18">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1227,7 +1189,7 @@
         <v>6.31</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:18">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1235,7 +1197,7 @@
         <v>7.84</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:18">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1243,7 +1205,7 @@
         <v>8.923</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:18">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1251,7 +1213,7 @@
         <v>3.112</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:18">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1259,7 +1221,7 @@
         <v>9.234</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:18">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1267,7 +1229,7 @@
         <v>6.224</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:18">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1275,7 +1237,7 @@
         <v>8.118</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:18">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1283,7 +1245,7 @@
         <v>6.405</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:18">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2784,14 +2746,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q201"/>
+  <dimension ref="A1:R201"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2831,8 +2793,11 @@
       <c r="Q1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:17">
+      <c r="R1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2878,8 +2843,12 @@
         <f t="array" ref="Q2">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,O2+J2,J2)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:17">
+      <c r="R2" cm="1">
+        <f t="array" ref="R2">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,0,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2887,7 +2856,7 @@
         <v>10.012</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:18">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2895,7 +2864,7 @@
         <v>11.888</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:18">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2903,7 +2872,7 @@
         <v>8.536</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:18">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2911,7 +2880,7 @@
         <v>6.597</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:18">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2919,7 +2888,7 @@
         <v>14.867</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:18">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2927,7 +2896,7 @@
         <v>10.012</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:18">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2935,7 +2904,7 @@
         <v>8.420999999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:18">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2943,7 +2912,7 @@
         <v>16.841</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:18">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2951,7 +2920,7 @@
         <v>13.451</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:18">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2959,7 +2928,7 @@
         <v>10.946</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:18">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2967,7 +2936,7 @@
         <v>14.702</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:18">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2975,7 +2944,7 @@
         <v>16.681</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:18">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2983,7 +2952,7 @@
         <v>10.012</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:18">
       <c r="A16">
         <v>15</v>
       </c>
@@ -4484,14 +4453,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q201"/>
+  <dimension ref="A1:R201"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4531,8 +4500,11 @@
       <c r="Q1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:17">
+      <c r="R1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4578,8 +4550,12 @@
         <f t="array" ref="Q2">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,O2+J2,J2)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:17">
+      <c r="R2" cm="1">
+        <f t="array" ref="R2">_xlfn.SEQUENCE(INT((P2-O2)/J2)+1,1,0,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
       <c r="A3">
         <v>2</v>
       </c>
@@ -4587,7 +4563,7 @@
         <v>16.247</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:18">
       <c r="A4">
         <v>3</v>
       </c>
@@ -4595,7 +4571,7 @@
         <v>4.406</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:18">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4603,7 +4579,7 @@
         <v>4.481</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:18">
       <c r="A6">
         <v>5</v>
       </c>
@@ -4611,7 +4587,7 @@
         <v>3.186</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:18">
       <c r="A7">
         <v>6</v>
       </c>
@@ -4619,7 +4595,7 @@
         <v>3.324</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:18">
       <c r="A8">
         <v>7</v>
       </c>
@@ -4627,7 +4603,7 @@
         <v>5.633</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:18">
       <c r="A9">
         <v>8</v>
       </c>
@@ -4635,7 +4611,7 @@
         <v>7.402</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:18">
       <c r="A10">
         <v>9</v>
       </c>
@@ -4643,7 +4619,7 @@
         <v>9.021000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:18">
       <c r="A11">
         <v>10</v>
       </c>
@@ -4651,7 +4627,7 @@
         <v>4.887</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:18">
       <c r="A12">
         <v>11</v>
       </c>
@@ -4659,7 +4635,7 @@
         <v>5.31</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:18">
       <c r="A13">
         <v>12</v>
       </c>
@@ -4667,7 +4643,7 @@
         <v>7.199</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:18">
       <c r="A14">
         <v>13</v>
       </c>
@@ -4675,7 +4651,7 @@
         <v>6.894</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:18">
       <c r="A15">
         <v>14</v>
       </c>
@@ -4683,7 +4659,7 @@
         <v>5.263</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:18">
       <c r="A16">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
created .bin file of macros
</commit_message>
<xml_diff>
--- a/100040000/output.xlsx
+++ b/100040000/output.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505" codeName="{37E998C4-C9E5-D4B9-71C8-EB1FF731991C}"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
@@ -1039,6 +1039,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:R201"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2746,6 +2747,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:R201"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -4453,6 +4455,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:R201"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>